<commit_message>
SHIA-SIA Nicosia: site validation script, updated investor pack and teaser, RTB sources
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/parks-for-sale/novikov/investor-pack/shia-sia-investor-model.xlsx
+++ b/parks-for-sale/novikov/investor-pack/shia-sia-investor-model.xlsx
@@ -418,7 +418,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>PARK-RTB-SIA-2026 | Lighthief Cyprus Ltd | 2026-06-15</v>
+        <v>PARK-RTB-SIA-2026 | Lighthief Cyprus Ltd | 2026-06-17</v>
       </c>
     </row>
     <row r="3"/>
@@ -491,12 +491,12 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Total CAPEX €3.94M | Gross revenue €680k | FCF €468k</v>
+        <v>Total CAPEX €4.03M | Gross revenue €706k | FCF €487k</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Cash-on-cash 11.9% | Simple payback 8.4 years</v>
+        <v>Cash-on-cash 12.1% | Simple payback 8.3 years</v>
       </c>
     </row>
   </sheetData>
@@ -553,7 +553,7 @@
         <v>Land</v>
       </c>
       <c r="B4" t="str">
-        <v>Plot 316, Sheet XXXIX/47, Sia, Larnaca District</v>
+        <v>Plot 316, Sheet 39/47, Sia, Larnaca District</v>
       </c>
       <c r="C4" t="str">
         <v>Lease executed 2025-05</v>
@@ -818,7 +818,7 @@
         <v>Solar MWp</v>
       </c>
       <c r="B2" s="1">
-        <v>3.2</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="3">
@@ -906,7 +906,7 @@
         <v>PV EPC €</v>
       </c>
       <c r="B13" s="1">
-        <v>2304000</v>
+        <v>2390400</v>
       </c>
     </row>
     <row r="14">
@@ -922,7 +922,7 @@
         <v>Total CAPEX €</v>
       </c>
       <c r="B15" s="1">
-        <v>3940342</v>
+        <v>4026742</v>
       </c>
     </row>
     <row r="16">
@@ -930,7 +930,7 @@
         <v>PV O&amp;M €/yr</v>
       </c>
       <c r="B16" s="1">
-        <v>25600</v>
+        <v>26560</v>
       </c>
     </row>
     <row r="17">
@@ -962,7 +962,7 @@
         <v>Insurance+admin €/yr</v>
       </c>
       <c r="B20" s="1">
-        <v>34702</v>
+        <v>35134</v>
       </c>
     </row>
   </sheetData>
@@ -1001,7 +1001,7 @@
         <v>Gross generation</v>
       </c>
       <c r="B2">
-        <v>4736</v>
+        <v>4914</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -1015,7 +1015,7 @@
         <v>Curtailed</v>
       </c>
       <c r="B3">
-        <v>2131</v>
+        <v>2211</v>
       </c>
       <c r="C3" t="str">
         <v>0 (stored)</v>
@@ -1029,13 +1029,13 @@
         <v>Uncurtailed solar export</v>
       </c>
       <c r="B4">
-        <v>2605</v>
+        <v>2702</v>
       </c>
       <c r="C4">
         <v>140.88</v>
       </c>
       <c r="D4">
-        <v>366992</v>
+        <v>380658</v>
       </c>
     </row>
     <row r="5">
@@ -1043,13 +1043,13 @@
         <v>BESS discharged</v>
       </c>
       <c r="B5">
-        <v>1607</v>
+        <v>1668</v>
       </c>
       <c r="C5">
         <v>195</v>
       </c>
       <c r="D5">
-        <v>313365</v>
+        <v>325260</v>
       </c>
     </row>
     <row r="6">
@@ -1063,7 +1063,7 @@
         <v/>
       </c>
       <c r="D6">
-        <v>680357</v>
+        <v>705918</v>
       </c>
     </row>
     <row r="7">
@@ -1077,7 +1077,7 @@
         <v/>
       </c>
       <c r="D7">
-        <v>0.8737681839511966</v>
+        <v>0.8738127544097694</v>
       </c>
     </row>
   </sheetData>
@@ -1164,7 +1164,7 @@
         <v>PV EPC</v>
       </c>
       <c r="B4">
-        <v>3.2</v>
+        <v>3.32</v>
       </c>
       <c r="C4" t="str">
         <v>MWp</v>
@@ -1173,7 +1173,7 @@
         <v>720000</v>
       </c>
       <c r="E4">
-        <v>2304000</v>
+        <v>2390400</v>
       </c>
       <c r="F4" t="str">
         <v>€0.72/Wp turnkey (Lighthief)</v>
@@ -1213,7 +1213,7 @@
         <v/>
       </c>
       <c r="E6">
-        <v>3940342</v>
+        <v>4026742</v>
       </c>
       <c r="F6" t="str">
         <v>Sum — ex VAT</v>
@@ -1315,10 +1315,10 @@
         <v>PV O&amp;M</v>
       </c>
       <c r="B2">
-        <v>25600</v>
+        <v>26560</v>
       </c>
       <c r="C2" t="str">
-        <v>€8000/MWp × 3.2 MWp</v>
+        <v>€8000/MWp × 3.32 MWp</v>
       </c>
       <c r="D2" t="str">
         <v>Shia-Sia scoped O&amp;M rate (investor pack assumption — confirm at NDA)</v>
@@ -1385,7 +1385,7 @@
         <v>Insurance + admin + SCADA</v>
       </c>
       <c r="B7">
-        <v>34702</v>
+        <v>35134</v>
       </c>
       <c r="C7" t="str">
         <v>0.5% CAPEX + €15000 admin</v>
@@ -1399,7 +1399,7 @@
         <v>Total OPEX Y1</v>
       </c>
       <c r="B8">
-        <v>97017</v>
+        <v>98409</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -1452,16 +1452,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>680357</v>
+        <v>705918</v>
       </c>
       <c r="C2" s="1">
-        <v>515304.30000000005</v>
+        <v>536917.2</v>
       </c>
       <c r="D2" s="1">
-        <v>46872</v>
+        <v>49466</v>
       </c>
       <c r="E2" s="1">
-        <v>468432.30000000005</v>
+        <v>487451.19999999995</v>
       </c>
       <c r="F2" s="2">
         <f>E2</f>
@@ -1473,16 +1473,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C3" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D3" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E3" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F3" s="2">
         <f>F2+E3</f>
@@ -1494,16 +1494,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C4" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D4" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E4" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F4" s="2">
         <f>F3+E4</f>
@@ -1515,16 +1515,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C5" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D5" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E5" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F5" s="2">
         <f>F4+E5</f>
@@ -1536,16 +1536,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C6" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D6" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E6" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F6" s="2">
         <f>F5+E6</f>
@@ -1557,16 +1557,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C7" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D7" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E7" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F7" s="2">
         <f>F6+E7</f>
@@ -1578,16 +1578,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C8" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D8" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E8" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F8" s="2">
         <f>F7+E8</f>
@@ -1599,16 +1599,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C9" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D9" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E9" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F9" s="2">
         <f>F8+E9</f>
@@ -1620,16 +1620,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C10" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D10" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E10" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F10" s="2">
         <f>F9+E10</f>
@@ -1641,16 +1641,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="1">
-        <v>676955</v>
+        <v>702388</v>
       </c>
       <c r="C11" s="1">
-        <v>512728</v>
+        <v>534233</v>
       </c>
       <c r="D11" s="1">
-        <v>46485</v>
+        <v>49063</v>
       </c>
       <c r="E11" s="1">
-        <v>466243</v>
+        <v>485170</v>
       </c>
       <c r="F11" s="2">
         <f>F10+E11</f>
@@ -1711,16 +1711,16 @@
         <v>195</v>
       </c>
       <c r="D2">
-        <v>680357</v>
+        <v>705918</v>
       </c>
       <c r="E2">
-        <v>468432.30000000005</v>
+        <v>487451.19999999995</v>
       </c>
       <c r="F2">
-        <v>0.11888112757725092</v>
+        <v>0.1210534968468305</v>
       </c>
       <c r="G2">
-        <v>8.411764090563352</v>
+        <v>8.260810518058014</v>
       </c>
     </row>
     <row r="3">
@@ -1734,16 +1734,16 @@
         <v>182.99</v>
       </c>
       <c r="D3">
-        <v>661057</v>
+        <v>685885</v>
       </c>
       <c r="E3">
-        <v>453668</v>
+        <v>472127</v>
       </c>
       <c r="F3">
-        <v>0.11513424469246579</v>
+        <v>0.11724776506664693</v>
       </c>
       <c r="G3">
-        <v>8.685513182208233</v>
+        <v>8.528947220713093</v>
       </c>
     </row>
     <row r="4">
@@ -1757,16 +1757,16 @@
         <v>165</v>
       </c>
       <c r="D4">
-        <v>577755</v>
+        <v>599460</v>
       </c>
       <c r="E4">
-        <v>389942</v>
+        <v>406011</v>
       </c>
       <c r="F4">
-        <v>0.09896133381315632</v>
+        <v>0.10082865999361271</v>
       </c>
       <c r="G4">
-        <v>10.104956769156399</v>
+        <v>9.91781503456803</v>
       </c>
     </row>
     <row r="5">
@@ -1780,16 +1780,16 @@
         <v>150</v>
       </c>
       <c r="D5">
-        <v>501550</v>
+        <v>520400</v>
       </c>
       <c r="E5">
-        <v>331645</v>
+        <v>345530</v>
       </c>
       <c r="F5">
-        <v>0.08416655204040664</v>
+        <v>0.08580882509979532</v>
       </c>
       <c r="G5">
-        <v>11.881204299778377</v>
+        <v>11.653812982953724</v>
       </c>
     </row>
     <row r="6">
@@ -1803,16 +1803,16 @@
         <v>165</v>
       </c>
       <c r="D6">
-        <v>650695</v>
+        <v>675116</v>
       </c>
       <c r="E6">
-        <v>445741</v>
+        <v>463887</v>
       </c>
       <c r="F6">
-        <v>0.11312228735475245</v>
+        <v>0.11520166924029401</v>
       </c>
       <c r="G6">
-        <v>8.839990981299657</v>
+        <v>8.680429776708744</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add HESS Psevdas BESS offer, new client packs, and financial updates.
HESS Psevdas: fix Package A commercial-quote arithmetic (consolidate battery/skid supply to a package-level subtotal tying to EUR 16,155,000); add offer generator/patch scripts.

New client offers: Ioannides Larnaca Mall, Evgeny tennis carport, UHE Ukraine hydro, German institutional PV+BESS, ETET Musa Lithuania.

Shia-Sia investor pack: model, teaser, sources and site-validation updates.

Financial: management pack, 12m transaction history, bank statement and shareholder-flow analysis (Jul 2026). Founder MOI-before-MOU letter drafts.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/parks-for-sale/novikov/investor-pack/shia-sia-investor-model.xlsx
+++ b/parks-for-sale/novikov/investor-pack/shia-sia-investor-model.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A23"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
@@ -429,88 +429,103 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Indicative 100% equity economics. All cited figures trace to Novikov DD package (May 2026),</v>
+        <v>Indicative 100% equity economics. This pack separates two domains:</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EAC connection OCR (ref 498000141), PVGIS yield run (Jun 2026), Lighthief EPC v4 pricing,</v>
+        <v xml:space="preserve">  PART A — SELLER PACKAGE (Novikov DD, May 2026): permits, EAC terms, land, seller PPA &amp; FM.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>and TSOC DAM sample (Oct 2025 – Feb 2026). Not an offer to sell securities.</v>
-      </c>
-    </row>
-    <row r="8"/>
+        <v xml:space="preserve">  PART B — LIGHTHIEF ANALYSIS: our E-W yield, BESS sizing, EPC pricing, merchant DAM revenue.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">  PART C — Seller financial model shown for comparison only (NOT the Lighthief stack).</v>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SHEETS</v>
+        <v>Sources: EAC OCR (498000141), PVGIS (Jun 2026), Lighthief EPC v4, TSOC DAM (Oct 2025–Feb 2026).</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>• Document_Sources — assumption registry with DD / market references</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>• Assumptions — editable inputs</v>
-      </c>
-    </row>
+        <v>Not an offer to sell securities.</v>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="str">
-        <v>• Revenue_Model — energy + DAM dispatch</v>
+        <v>SHEETS</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>• CAPEX — line items with unit rates</v>
+        <v>• Document_Sources — assumption registry with DD / market references</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>• OPEX — annual operating costs</v>
+        <v>• Assumptions — editable inputs</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>• P_and_L — 10-year simplified cash flow</v>
+        <v>• Revenue_Model — energy + DAM dispatch</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>• DAM_Sensitivity — merchant price scenarios</v>
-      </c>
-    </row>
-    <row r="17"/>
+        <v>• CAPEX — line items with unit rates</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>• OPEX — annual operating costs</v>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>KEY OUTPUTS (Y1)</v>
+        <v>• P_and_L — 10-year simplified cash flow</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Total CAPEX €4.03M | Gross revenue €706k | FCF €487k</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Cash-on-cash 12.1% | Simple payback 8.3 years</v>
+        <v>• DAM_Sensitivity — merchant price scenarios</v>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>KEY OUTPUTS (Y1)</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Total CAPEX €5.10M | Gross revenue €661k | FCF €460k</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Cash-on-cash 9.0% | Simple payback 11.1 years</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C30"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="55.83203125" customWidth="1"/>
   </cols>
@@ -528,87 +543,87 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CERA licence</v>
+        <v>── PART A · SELLER-PROVIDED (Novikov DD, as received) ──</v>
       </c>
       <c r="B2" t="str">
-        <v>E3511</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>DD package — CERA E3511 Apr 2025</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Town planning</v>
+        <v>CERA licence</v>
       </c>
       <c r="B3" t="str">
-        <v>3.32 MWp</v>
+        <v>E3511</v>
       </c>
       <c r="C3" t="str">
-        <v>Issued 2025-05-05</v>
+        <v>DD package — CERA E3511 Apr 2025</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Land</v>
+        <v>Town planning</v>
       </c>
       <c r="B4" t="str">
-        <v>Plot 316, Sheet 39/47, Sia, Larnaca District</v>
+        <v>3.32 MWp</v>
       </c>
       <c r="C4" t="str">
-        <v>Lease executed 2025-05</v>
+        <v>Issued 2025-05-05</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>EAC connection ref</v>
+        <v>Land</v>
       </c>
       <c r="B5" t="str">
-        <v>498000141</v>
+        <v>Plot 316, Sheet 39/47, Sia, Larnaca District</v>
       </c>
       <c r="C5" t="str">
-        <v>EAC connection/498000141_Grid_Connection_Terms_SIA.pdf</v>
+        <v>Lease executed 2025-05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EAC grid works (prelim.)</v>
-      </c>
-      <c r="B6">
-        <v>83842.14</v>
+        <v>EAC connection ref</v>
+      </c>
+      <c r="B6" t="str">
+        <v>498000141</v>
       </c>
       <c r="C6" t="str">
-        <v>OCR 498000141 — NOT BINDING</v>
+        <v>EAC connection/498000141_Grid_Connection_Terms_SIA.pdf</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>EAC deposit paid</v>
+        <v>EAC grid works (prelim.)</v>
       </c>
       <c r="B7">
-        <v>4988.61</v>
+        <v>83842.14</v>
       </c>
       <c r="C7" t="str">
-        <v>Paid 2022-02-22</v>
+        <v>OCR 498000141 — NOT BINDING</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>EAC annual telecom</v>
+        <v>EAC deposit paid</v>
       </c>
       <c r="B8">
-        <v>180</v>
+        <v>4988.61</v>
       </c>
       <c r="C8" t="str">
-        <v>Connection terms OCR</v>
+        <v>Paid 2022-02-22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EAC substation sublease</v>
+        <v>EAC annual telecom</v>
       </c>
       <c r="B9">
-        <v>10</v>
+        <v>180</v>
       </c>
       <c r="C9" t="str">
         <v>Connection terms OCR</v>
@@ -616,183 +631,238 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>AC export limit</v>
-      </c>
-      <c r="B10" t="str">
-        <v>2.7 MW</v>
+        <v>EAC substation sublease</v>
+      </c>
+      <c r="B10">
+        <v>10</v>
       </c>
       <c r="C10" t="str">
-        <v>Huawei SUN2000-150K — 3 × 330 kW (per DD technical summary)</v>
+        <v>Connection terms OCR</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PV layout</v>
+        <v>AC export limit</v>
       </c>
       <c r="B11" t="str">
-        <v>Bifacial east–west 10° (50% aspect −90° + 50% aspect +90°)</v>
+        <v>2.7 MW</v>
       </c>
       <c r="C11" t="str">
-        <v>PVGIS API v5.2 2026-06-15</v>
+        <v>Huawei SUN2000-150K — 3 × 330 kW (per DD technical summary)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>PV yield (model)</v>
-      </c>
-      <c r="B12">
-        <v>1480</v>
+        <v>Seller PPA (not in LH base)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>$0.16/kWh</v>
       </c>
       <c r="C12" t="str">
-        <v>scripts/pvgis-park-yield.py</v>
+        <v>Draft v2 — January 2026, not executed</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Curtailment base</v>
-      </c>
-      <c r="B13" t="str">
-        <v>45%</v>
+        <v>Seller FM total CAPEX</v>
+      </c>
+      <c r="B13">
+        <v>4780000</v>
       </c>
       <c r="C13" t="str">
-        <v>E-W flatter profile vs 50% south baseline</v>
+        <v>FM_3,2MW_250126_BESS.xlsx — comparison only</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>BESS size</v>
+        <v>Seller equity IRR</v>
       </c>
       <c r="B14" t="str">
-        <v>2.5 MW / 7.5 MWh</v>
+        <v>29.7%</v>
       </c>
       <c r="C14" t="str">
-        <v>3h — energy cap 280 cycle days/yr</v>
+        <v>Seller model — south-facing, levered</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Solar DAM price</v>
-      </c>
-      <c r="B15">
-        <v>140.88</v>
+        <v>── PART B · LIGHTHIEF ANALYSIS (our EPC + merchant model) ──</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
       </c>
       <c r="C15" t="str">
-        <v>134 TSOC day-ahead days (1 Oct 2025 – 11 Feb 2026), 6,432 half-hourly prints</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>BESS discharge price</v>
-      </c>
-      <c r="B16">
-        <v>195</v>
+        <v>PV layout</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Bifacial east–west 10° (50% aspect −90° + 50% aspect +90°)</v>
       </c>
       <c r="C16" t="str">
-        <v>Measured evening avg €182.99; blended conservative</v>
+        <v>PVGIS API v5.2 2026-06-15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>BESS RTE</v>
+        <v>PV yield (model)</v>
       </c>
       <c r="B17">
-        <v>0.8632</v>
+        <v>1480</v>
       </c>
       <c r="C17" t="str">
-        <v>Galascope 2.5 MW 2025 actual</v>
+        <v>scripts/pvgis-park-yield.py</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>BESS capture</v>
-      </c>
-      <c r="B18" t="str">
-        <v>87.4%</v>
+        <v>South 15° reference (not used)</v>
+      </c>
+      <c r="B18">
+        <v>1633</v>
       </c>
       <c r="C18" t="str">
-        <v>Curtailed energy × cap at MWh×280 days</v>
+        <v>Permit layout comparison only</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>PV EPC rate</v>
-      </c>
-      <c r="B19">
-        <v>720000</v>
+        <v>Curtailment base</v>
+      </c>
+      <c r="B19" t="str">
+        <v>45%</v>
       </c>
       <c r="C19" t="str">
-        <v>lib/deals/rtb-deal-types.ts LH_EPC + RTB_COSTS; Lighthief-EPC-Confirmed-Adders-v4-Feb2026.xlsx</v>
+        <v>E-W flatter profile vs 50% south baseline</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BESS EPC rate</v>
-      </c>
-      <c r="B20">
-        <v>127000</v>
+        <v>BESS size</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2.5 MW / 7.5 MWh</v>
       </c>
       <c r="C20" t="str">
-        <v>lib/deals/rtb-deal-types.ts LH_EPC + RTB_COSTS; Lighthief-EPC-Confirmed-Adders-v4-Feb2026.xlsx</v>
+        <v>3h — energy cap 280 cycle days/yr</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>RTB acquisition</v>
+        <v>Solar DAM price</v>
       </c>
       <c r="B21">
-        <v>600000</v>
+        <v>140.88</v>
       </c>
       <c r="C21" t="str">
-        <v>RTB_COSTS.withConnectionTerms</v>
+        <v>134 TSOC day-ahead days (1 Oct 2025 – 11 Feb 2026), 6,432 half-hourly prints</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>PV O&amp;M</v>
+        <v>BESS discharge price</v>
       </c>
       <c r="B22">
-        <v>8000</v>
+        <v>182.99</v>
       </c>
       <c r="C22" t="str">
-        <v>Shia-Sia scoped O&amp;M rate (investor pack assumption — confirm at NDA)</v>
+        <v>TSOC evening avg 17–21h — 134 TSOC day-ahead days (1 Oct 2025 – 11 Feb 2026), 6,432 half-hourly prints</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Land lease</v>
+        <v>BESS RTE</v>
       </c>
       <c r="B23">
-        <v>18000</v>
+        <v>0.8632</v>
       </c>
       <c r="C23" t="str">
-        <v>INDICATIVE — executed lease May 2025 on file; annual rent not OCR’d from deed</v>
+        <v>Galascope 2.5 MW 2025 actual</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Seller PPA (not in base)</v>
+        <v>BESS capture</v>
       </c>
       <c r="B24" t="str">
-        <v>$0.16/kWh</v>
+        <v>87.4%</v>
       </c>
       <c r="C24" t="str">
-        <v>Draft v2 — January 2026, not executed</v>
+        <v>Curtailed energy × cap at MWh×280 days</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Seller FM total CAPEX</v>
+        <v>PV EPC rate</v>
       </c>
       <c r="B25">
-        <v>4780000</v>
+        <v>720000</v>
       </c>
       <c r="C25" t="str">
-        <v>FM_3,2MW_250126_BESS.xlsx — comparison only</v>
+        <v>lib/deals/rtb-deal-types.ts LH_EPC; Lighthief-EPC-Confirmed-Adders-v4-Feb2026.xlsx</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>BESS EPC rate</v>
+      </c>
+      <c r="B26">
+        <v>127000</v>
+      </c>
+      <c r="C26" t="str">
+        <v>lib/deals/rtb-deal-types.ts LH_EPC; Lighthief-EPC-Confirmed-Adders-v4-Feb2026.xlsx</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>RTB acquisition</v>
+      </c>
+      <c r="B27">
+        <v>1760000</v>
+      </c>
+      <c r="C27" t="str">
+        <v>€550k/MWp × 3.2 MWp (RTB incl. connection terms)</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>PV O&amp;M</v>
+      </c>
+      <c r="B28">
+        <v>8000</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Shia-Sia scoped O&amp;M rate (investor pack assumption — confirm at NDA)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Land lease</v>
+      </c>
+      <c r="B29">
+        <v>18000</v>
+      </c>
+      <c r="C29" t="str">
+        <v>INDICATIVE — executed lease May 2025 on file; annual rent not OCR’d from deed</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>LH total CAPEX</v>
+      </c>
+      <c r="B30">
+        <v>5100342</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Lighthief EPC stack (ex VAT)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -818,7 +888,7 @@
         <v>Solar MWp</v>
       </c>
       <c r="B2" s="1">
-        <v>3.32</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="3">
@@ -866,7 +936,7 @@
         <v>BESS discharge €/MWh</v>
       </c>
       <c r="B8" s="1">
-        <v>195</v>
+        <v>182.99</v>
       </c>
     </row>
     <row r="9">
@@ -890,7 +960,7 @@
         <v>RTB acquisition €</v>
       </c>
       <c r="B11" s="1">
-        <v>600000</v>
+        <v>1760000</v>
       </c>
     </row>
     <row r="12">
@@ -906,7 +976,7 @@
         <v>PV EPC €</v>
       </c>
       <c r="B13" s="1">
-        <v>2390400</v>
+        <v>2304000</v>
       </c>
     </row>
     <row r="14">
@@ -922,7 +992,7 @@
         <v>Total CAPEX €</v>
       </c>
       <c r="B15" s="1">
-        <v>4026742</v>
+        <v>5100342</v>
       </c>
     </row>
     <row r="16">
@@ -930,7 +1000,7 @@
         <v>PV O&amp;M €/yr</v>
       </c>
       <c r="B16" s="1">
-        <v>26560</v>
+        <v>25600</v>
       </c>
     </row>
     <row r="17">
@@ -962,7 +1032,7 @@
         <v>Insurance+admin €/yr</v>
       </c>
       <c r="B20" s="1">
-        <v>35134</v>
+        <v>40502</v>
       </c>
     </row>
   </sheetData>
@@ -1001,7 +1071,7 @@
         <v>Gross generation</v>
       </c>
       <c r="B2">
-        <v>4914</v>
+        <v>4736</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -1015,7 +1085,7 @@
         <v>Curtailed</v>
       </c>
       <c r="B3">
-        <v>2211</v>
+        <v>2131</v>
       </c>
       <c r="C3" t="str">
         <v>0 (stored)</v>
@@ -1029,13 +1099,13 @@
         <v>Uncurtailed solar export</v>
       </c>
       <c r="B4">
-        <v>2702</v>
+        <v>2605</v>
       </c>
       <c r="C4">
         <v>140.88</v>
       </c>
       <c r="D4">
-        <v>380658</v>
+        <v>366992</v>
       </c>
     </row>
     <row r="5">
@@ -1043,13 +1113,13 @@
         <v>BESS discharged</v>
       </c>
       <c r="B5">
-        <v>1668</v>
+        <v>1607</v>
       </c>
       <c r="C5">
-        <v>195</v>
+        <v>182.99</v>
       </c>
       <c r="D5">
-        <v>325260</v>
+        <v>294065</v>
       </c>
     </row>
     <row r="6">
@@ -1063,7 +1133,7 @@
         <v/>
       </c>
       <c r="D6">
-        <v>705918</v>
+        <v>661057</v>
       </c>
     </row>
     <row r="7">
@@ -1077,7 +1147,7 @@
         <v/>
       </c>
       <c r="D7">
-        <v>0.8738127544097694</v>
+        <v>0.8737681839511966</v>
       </c>
     </row>
   </sheetData>
@@ -1089,7 +1159,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -1124,19 +1194,19 @@
         <v>RTB acquisition (incl. connection terms issued)</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="C2" t="str">
-        <v>lump sum</v>
+        <v>MWp</v>
       </c>
       <c r="D2">
-        <v>600000</v>
+        <v>550000</v>
       </c>
       <c r="E2">
-        <v>600000</v>
+        <v>1760000</v>
       </c>
       <c r="F2" t="str">
-        <v>RTB_COSTS.withConnectionTerms — DD May 2026</v>
+        <v>€550k/MWp ready-to-build</v>
       </c>
     </row>
     <row r="3">
@@ -1164,7 +1234,7 @@
         <v>PV EPC</v>
       </c>
       <c r="B4">
-        <v>3.32</v>
+        <v>3.2</v>
       </c>
       <c r="C4" t="str">
         <v>MWp</v>
@@ -1173,7 +1243,7 @@
         <v>720000</v>
       </c>
       <c r="E4">
-        <v>2390400</v>
+        <v>2304000</v>
       </c>
       <c r="F4" t="str">
         <v>€0.72/Wp turnkey (Lighthief)</v>
@@ -1201,7 +1271,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Total project CAPEX</v>
+        <v>Total project CAPEX (LIGHTHIEF stack)</v>
       </c>
       <c r="B6" t="str">
         <v/>
@@ -1213,7 +1283,7 @@
         <v/>
       </c>
       <c r="E6">
-        <v>4026742</v>
+        <v>5100342</v>
       </c>
       <c r="F6" t="str">
         <v>Sum — ex VAT</v>
@@ -1241,7 +1311,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Seller comparison (NOT in Lighthief stack)</v>
+        <v>── SELLER MODEL (comparison only, NOT Lighthief) ──</v>
       </c>
       <c r="B8" t="str">
         <v/>
@@ -1252,36 +1322,56 @@
       <c r="D8" t="str">
         <v/>
       </c>
-      <c r="E8">
-        <v>4780000</v>
+      <c r="E8" t="str">
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>FM_3,2MW_250126_BESS.xlsx</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Seller total CAPEX</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9">
+        <v>4780000</v>
+      </c>
+      <c r="F9" t="str">
+        <v>FM_3,2MW_250126_BESS.xlsx</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v xml:space="preserve">  of which seller dev/licence</v>
       </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9">
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10">
         <v>1600000</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F10" t="str">
         <v>Novikov embedded development</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1315,10 +1405,10 @@
         <v>PV O&amp;M</v>
       </c>
       <c r="B2">
-        <v>26560</v>
+        <v>25600</v>
       </c>
       <c r="C2" t="str">
-        <v>€8000/MWp × 3.32 MWp</v>
+        <v>€8000/MWp × 3.2 MWp</v>
       </c>
       <c r="D2" t="str">
         <v>Shia-Sia scoped O&amp;M rate (investor pack assumption — confirm at NDA)</v>
@@ -1385,7 +1475,7 @@
         <v>Insurance + admin + SCADA</v>
       </c>
       <c r="B7">
-        <v>35134</v>
+        <v>40502</v>
       </c>
       <c r="C7" t="str">
         <v>0.5% CAPEX + €15000 admin</v>
@@ -1399,7 +1489,7 @@
         <v>Total OPEX Y1</v>
       </c>
       <c r="B8">
-        <v>98409</v>
+        <v>102817</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -1452,16 +1542,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>705918</v>
+        <v>661057</v>
       </c>
       <c r="C2" s="1">
-        <v>536917.2</v>
+        <v>492134.30000000005</v>
       </c>
       <c r="D2" s="1">
-        <v>49466</v>
+        <v>31796</v>
       </c>
       <c r="E2" s="1">
-        <v>487451.19999999995</v>
+        <v>460338.30000000005</v>
       </c>
       <c r="F2" s="2">
         <f>E2</f>
@@ -1473,16 +1563,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C3" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D3" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E3" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F3" s="2">
         <f>F2+E3</f>
@@ -1494,16 +1584,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C4" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D4" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E4" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F4" s="2">
         <f>F3+E4</f>
@@ -1515,16 +1605,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C5" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D5" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E5" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F5" s="2">
         <f>F4+E5</f>
@@ -1536,16 +1626,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C6" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D6" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E6" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F6" s="2">
         <f>F5+E6</f>
@@ -1557,16 +1647,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C7" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D7" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E7" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F7" s="2">
         <f>F6+E7</f>
@@ -1578,16 +1668,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C8" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D8" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E8" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F8" s="2">
         <f>F7+E8</f>
@@ -1599,16 +1689,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C9" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D9" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E9" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F9" s="2">
         <f>F8+E9</f>
@@ -1620,16 +1710,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C10" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D10" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E10" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F10" s="2">
         <f>F9+E10</f>
@@ -1641,16 +1731,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="1">
-        <v>702388</v>
+        <v>657752</v>
       </c>
       <c r="C11" s="1">
-        <v>534233</v>
+        <v>489674</v>
       </c>
       <c r="D11" s="1">
-        <v>49063</v>
+        <v>31427</v>
       </c>
       <c r="E11" s="1">
-        <v>485170</v>
+        <v>458247</v>
       </c>
       <c r="F11" s="2">
         <f>F10+E11</f>
@@ -1702,48 +1792,48 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Base (model)</v>
+        <v>Base (TSOC evening avg)</v>
       </c>
       <c r="B2">
         <v>140.88</v>
       </c>
       <c r="C2">
-        <v>195</v>
+        <v>182.99</v>
       </c>
       <c r="D2">
-        <v>705918</v>
+        <v>661057</v>
       </c>
       <c r="E2">
-        <v>487451.19999999995</v>
+        <v>460338.30000000005</v>
       </c>
       <c r="F2">
-        <v>0.1210534968468305</v>
+        <v>0.09025635927943657</v>
       </c>
       <c r="G2">
-        <v>8.260810518058014</v>
+        <v>11.079551712295066</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TSOC measured BESS only</v>
+        <v>Upside blended €195 BESS</v>
       </c>
       <c r="B3">
         <v>140.88</v>
       </c>
       <c r="C3">
-        <v>182.99</v>
+        <v>195</v>
       </c>
       <c r="D3">
-        <v>685885</v>
+        <v>680357</v>
       </c>
       <c r="E3">
-        <v>472127</v>
+        <v>475102</v>
       </c>
       <c r="F3">
-        <v>0.11724776506664693</v>
+        <v>0.09315106712451833</v>
       </c>
       <c r="G3">
-        <v>8.528947220713093</v>
+        <v>10.735250071405673</v>
       </c>
     </row>
     <row r="4">
@@ -1757,16 +1847,16 @@
         <v>165</v>
       </c>
       <c r="D4">
-        <v>599460</v>
+        <v>577755</v>
       </c>
       <c r="E4">
-        <v>406011</v>
+        <v>396612</v>
       </c>
       <c r="F4">
-        <v>0.10082865999361271</v>
+        <v>0.07776174617309976</v>
       </c>
       <c r="G4">
-        <v>9.91781503456803</v>
+        <v>12.859793525906333</v>
       </c>
     </row>
     <row r="5">
@@ -1780,16 +1870,16 @@
         <v>150</v>
       </c>
       <c r="D5">
-        <v>520400</v>
+        <v>501550</v>
       </c>
       <c r="E5">
-        <v>345530</v>
+        <v>338315</v>
       </c>
       <c r="F5">
-        <v>0.08580882509979532</v>
+        <v>0.06633182637556462</v>
       </c>
       <c r="G5">
-        <v>11.653812982953724</v>
+        <v>15.075719373956224</v>
       </c>
     </row>
     <row r="6">
@@ -1803,16 +1893,16 @@
         <v>165</v>
       </c>
       <c r="D6">
-        <v>675116</v>
+        <v>650695</v>
       </c>
       <c r="E6">
-        <v>463887</v>
+        <v>452411</v>
       </c>
       <c r="F6">
-        <v>0.11520166924029401</v>
+        <v>0.08870199292518031</v>
       </c>
       <c r="G6">
-        <v>8.680429776708744</v>
+        <v>11.27370385965843</v>
       </c>
     </row>
   </sheetData>

</xml_diff>